<commit_message>
Shopping list: RdestGrabber details, one BNC-RCA adapter
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAtxAoTbpkfDbjG9oAM3Vj
</commit_message>
<xml_diff>
--- a/docs/shopping-list.xlsx
+++ b/docs/shopping-list.xlsx
@@ -79,7 +79,7 @@
     <t xml:space="preserve">Antena 5.8 GHz dookólna (ta sama polaryzacja)</t>
   </si>
   <si>
-    <t xml:space="preserve">Grabber USB CVBS „no blue screen” (rdest.io)</t>
+    <t xml:space="preserve">RdestGrabber – grabber USB CVBS „no blue screen” (rdest.io, wejście RCA, UVC)</t>
   </si>
   <si>
     <t xml:space="preserve">Para pasywnych balunów wideo CCTV (BNC ↔ skrętka)</t>
@@ -88,7 +88,7 @@
     <t xml:space="preserve">Gniazdo BNC do lutowania (wyjście wideo SteadyView)</t>
   </si>
   <si>
-    <t xml:space="preserve">Przejściówka BNC ↔ RCA (zależy od złącza grabbera)</t>
+    <t xml:space="preserve">Przejściówka BNC (gniazdo) ↔ RCA (wtyk): balun → wejście RCA grabbera</t>
   </si>
   <si>
     <t xml:space="preserve">Przewód ekranowany cienki (mini-koncentryk), 0,5 m</t>
@@ -323,16 +323,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -344,11 +348,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -364,7 +368,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -642,448 +646,448 @@
   <dimension ref="A1:C47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="B6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="B7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="C8" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="C9" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="C10" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="B11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="B12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="C13" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+      <c r="B16" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="B17" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="B18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+      <c r="B19" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="B20" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
+      <c r="B21" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
+      <c r="B22" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="B23" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="8" t="n">
+      <c r="B25" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
+      <c r="C25" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
+      <c r="B26" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="8" t="n">
+      <c r="B27" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+      <c r="C27" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
+      <c r="B28" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
+      <c r="B29" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="s">
+      <c r="B30" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
+      <c r="B31" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
+      <c r="B32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
+      <c r="B33" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="s">
+      <c r="B34" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B35" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
+      <c r="B35" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B36" s="8" t="n">
+      <c r="B36" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C36" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
+      <c r="C36" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
+      <c r="B37" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="6"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="s">
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="s">
+      <c r="B39" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B40" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
+      <c r="B40" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10" t="s">
+      <c r="B41" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="11" t="str">
+      <c r="B43" s="12" t="str">
         <f aca="false">COUNTIF(C6:C41,"TAK")&amp;" / "&amp;(COUNTIF(C6:C41,"TAK")+COUNTIF(C6:C41,"NIE"))</f>
         <v>0 / 33</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="10" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B44" s="11" t="n">
+      <c r="B44" s="12" t="n">
         <f aca="false">COUNTIF(C6:C41,"NIE")</f>
         <v>33</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 3D-printable mast enclosure, switch ELRS module to Radiomaster Nomad
Parametric OpenSCAD enclosure (box, lid with gasket groove, mounting
plate, V-groove mast bracket for velcro straps / zip ties) sized for a
180x180 bed, with STL exports and previews. All openings are in the
bottom wall. Docs and shopping list updated for the Nomad (6-16.8 V via
XT30, so a 12 V converter is needed again; EU868/2.4 GHz power limits).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAtxAoTbpkfDbjG9oAM3Vj
</commit_message>
<xml_diff>
--- a/docs/shopping-list.xlsx
+++ b/docs/shopping-list.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="53">
   <si>
     <t xml:space="preserve">Lista zakupów – FPV GCS z masztem (weakgcs)</t>
   </si>
@@ -49,10 +49,16 @@
     <t xml:space="preserve">NIE</t>
   </si>
   <si>
-    <t xml:space="preserve">Moduł ELRS TX 2.4 GHz, firmware EU/LBT (np. Radiomaster Ranger Micro/Nano) – jeśli nie mam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Przetwornica step-down 5 V ≥3 A, wejście do 28 V (ESP32+ELRS i osobno SteadyView)</t>
+    <t xml:space="preserve">Radiomaster Nomad Dual 1W Gemini Xrossband (ELRS 2.4 GHz + 868 MHz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Przetwornica step-down 5 V, wejście do 28 V (ESP32 i osobno SteadyView)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Przetwornica step-down 12 V ≥2 A (XL4015) – zasilanie Nomada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wtyk XT30 z przewodem (zasilanie Nomada)</t>
   </si>
   <si>
     <t xml:space="preserve">Kondensator low-ESR 470–1000 µF / 35 V</t>
@@ -133,10 +139,22 @@
     <t xml:space="preserve">Podstawa/statyw lub szpilka + odciągi</t>
   </si>
   <si>
-    <t xml:space="preserve">Puszka hermetyczna IP65 ~150×100×70 mm + dławiki kablowe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Przedłużka antenowa SMA low-loss ≤20 cm (sprawdzić SMA vs RP-SMA)</t>
+    <t xml:space="preserve">Filament ASA lub PETG na obudowę (ok. 300 g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wtopki gwintowane M3 (heat-set)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wkręty M3×8 (nierdzewne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sznur uszczelniający Ø2 mm (silikon/EPDM) – metry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dławik kablowy PG9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Przedłużka SMA bulkhead (gniazdo panelowe ↔ wtyk), RG316, 10–15 cm</t>
   </si>
   <si>
     <t xml:space="preserve">Uchwyty anten, obejmy, opaski, rzepy</t>
@@ -160,7 +178,7 @@
     <t xml:space="preserve">Pozostało do kupienia</t>
   </si>
   <si>
-    <t xml:space="preserve">Nie kupuję: osobnego VRX (mam SteadyView V3.3), przetwornicy 12 V, injectora PoE, drugiego grabbera.</t>
+    <t xml:space="preserve">Nie kupuję: osobnego VRX (mam SteadyView V3.3), gotowej puszki (obudowa z druku 3D), injectora PoE, drugiego grabbera.</t>
   </si>
   <si>
     <t xml:space="preserve">Pary skrętki: pomarańczowa+zielona = Ethernet, niebieska = wideo, brązowa = 24 V. Nie podawać 24 V do RJ45 płytki ESP32.</t>
@@ -643,7 +661,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="78"/>
@@ -717,7 +735,7 @@
         <v>10</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>7</v>
@@ -728,7 +746,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>7</v>
@@ -739,7 +757,7 @@
         <v>12</v>
       </c>
       <c r="B11" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>7</v>
@@ -750,7 +768,7 @@
         <v>13</v>
       </c>
       <c r="B12" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>7</v>
@@ -761,40 +779,40 @@
         <v>14</v>
       </c>
       <c r="B13" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
+      <c r="B14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>7</v>
-      </c>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
@@ -874,40 +892,40 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
+      <c r="B24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="9" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>7</v>
-      </c>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
         <v>28</v>
       </c>
       <c r="B27" s="9" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C27" s="10" t="s">
         <v>7</v>
@@ -929,7 +947,7 @@
         <v>30</v>
       </c>
       <c r="B29" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C29" s="10" t="s">
         <v>7</v>
@@ -1006,7 +1024,7 @@
         <v>37</v>
       </c>
       <c r="B36" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C36" s="10" t="s">
         <v>7</v>
@@ -1024,18 +1042,22 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
+      <c r="B38" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B39" s="9" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C39" s="10" t="s">
         <v>7</v>
@@ -1063,42 +1085,104 @@
         <v>7</v>
       </c>
     </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B43" s="12" t="str">
-        <f aca="false">COUNTIF(C6:C41,"TAK")&amp;" / "&amp;(COUNTIF(C6:C41,"TAK")+COUNTIF(C6:C41,"NIE"))</f>
-        <v>0 / 33</v>
+      <c r="A43" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B44" s="12" t="n">
-        <f aca="false">COUNTIF(C6:C41,"NIE")</f>
-        <v>33</v>
+      <c r="A44" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>45</v>
+      <c r="A46" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B46" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
-        <v>46</v>
+      <c r="A47" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B47" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B49" s="12" t="str">
+        <f aca="false">COUNTIF(C6:C47,"TAK")&amp;" / "&amp;(COUNTIF(C6:C47,"TAK")+COUNTIF(C6:C47,"NIE"))</f>
+        <v>0 / 39</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B50" s="12" t="n">
+        <f aca="false">COUNTIF(C6:C47,"NIE")</f>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A6:C41">
+  <conditionalFormatting sqref="A6:C47">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$C6="TAK"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6:C13 C15:C23 C25:C37 C39:C41" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6:C15 C17:C25 C27:C43 C45:C47" type="list">
       <formula1>"TAK,NIE"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>